<commit_message>
Different PDFs and commands in Git Excel and initialized highlighting Progit book
</commit_message>
<xml_diff>
--- a/Git/Git_Commands.xlsx
+++ b/Git/Git_Commands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IDM\Documents\Books\Git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41394F9-22E8-4697-9D54-15B1D39CAC27}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6EE7E0-C4B0-4C26-90C6-2F7D68E4CE70}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,12 +25,133 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>Git Commands</t>
   </si>
   <si>
     <t>What do they do ?</t>
+  </si>
+  <si>
+    <t>$ git config --list --show-origin</t>
+  </si>
+  <si>
+    <t>You can view all of your settings and where they are coming from</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ git config --global user.name "John Doe"
+</t>
+  </si>
+  <si>
+    <t>$ git config --global user.email johndoe@example.com</t>
+  </si>
+  <si>
+    <t>Sets your name globally</t>
+  </si>
+  <si>
+    <t>Set your email globally</t>
+  </si>
+  <si>
+    <t>Remarks(Explanation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If you want to override this with a different name or email address for specific projects, you can run the command without the --global option when you’re in that project.</t>
+  </si>
+  <si>
+    <t>$ git config --global core.editor "'C:/Program Files/Notepad++/notepad++.exe' -multiInst -notabbar -nosession -noPlugin"</t>
+  </si>
+  <si>
+    <t>you can configure the default text editor that will be used when Git needs you to type in a message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If you want to override this with a different editor for specific projects, you can run the command without the --global option when you’re in that project.</t>
+  </si>
+  <si>
+    <t>$ git config --global init.defaultBranch main</t>
+  </si>
+  <si>
+    <t>By default Git will create a branch called master when you create a new repository with git init. From Git version 2.28 onwards, you can set a different name for the initial branch.</t>
+  </si>
+  <si>
+    <t>To set main as the default branch name</t>
+  </si>
+  <si>
+    <t>$ git config --list</t>
+  </si>
+  <si>
+    <t>to list all the settings Git can find at that point</t>
+  </si>
+  <si>
+    <t>You may see keys more than once, because Git reads the same key from different files ([path]/etc/gitconfig and ~/.gitconfig, for example). In this case, Git uses the last value for each
+unique key it sees.</t>
+  </si>
+  <si>
+    <t>$ git config --show-origin rerere.autoUpdate</t>
+  </si>
+  <si>
+    <t>origin for a key(here key is rerere.autoupdate)</t>
+  </si>
+  <si>
+    <t>Since Git might read the same configuration variable value from more than one file, it’s possible that you have an unexpected value for one of these values and you don’t know why. In cases like that, you can query Git as to the origin for that value, and it will tell you which configuration file had the final say in setting that value</t>
+  </si>
+  <si>
+    <t>$ git help &lt;verb&gt;
+$ git &lt;verb&gt; --help 
+$ man git - &lt;verb&gt;</t>
+  </si>
+  <si>
+    <t>to get the comprehensive manual page (manpage) help for any of the Git commands</t>
+  </si>
+  <si>
+    <t>$ git init</t>
+  </si>
+  <si>
+    <t>Initializes a new local git repository</t>
+  </si>
+  <si>
+    <t>$ git clone https://github.com/libgit2/libgit2 mylibgit</t>
+  </si>
+  <si>
+    <t>Clones the remote directory in mylibgit folder</t>
+  </si>
+  <si>
+    <t>$ git status</t>
+  </si>
+  <si>
+    <t>which files are in which state is</t>
+  </si>
+  <si>
+    <t>$ git add CONTRIBUTING.md</t>
+  </si>
+  <si>
+    <t>git add is a multipurpose command — you use it to begin tracking new files, to stage files, and to do other things like marking merge-conflicted files as resolved</t>
+  </si>
+  <si>
+    <t>to add file in satging area</t>
+  </si>
+  <si>
+    <t>$ git commit</t>
+  </si>
+  <si>
+    <t>Doing so launches your editor of choice.</t>
+  </si>
+  <si>
+    <t>simplest way to commit</t>
+  </si>
+  <si>
+    <t>$ git commit -m "Story 182: fix benchmarks for speed"</t>
+  </si>
+  <si>
+    <t>Alternatively, you can type your commit message inline with the commit command by specifying it after a -m flag</t>
+  </si>
+  <si>
+    <t>$ git commit -a -m 'Add new benchmarks'</t>
+  </si>
+  <si>
+    <t>Adding the -a option to the git commit command makes Git automatically stage every file that is already tracked before doing the commit, letting you skip the git add part</t>
+  </si>
+  <si>
+    <t>skipping git add coomand</t>
   </si>
 </sst>
 </file>
@@ -94,9 +215,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -378,22 +523,174 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.42578125" customWidth="1"/>
-    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="1" max="1" width="111.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="163.5703125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="8"/>
+    </row>
+    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:C4"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Started Topic Wise sheet till GIT Aliases on Oct 04, 2022
</commit_message>
<xml_diff>
--- a/Git/Git_Commands.xlsx
+++ b/Git/Git_Commands.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Books\Git\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Books\Git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD545D49-33A6-4F67-BD41-6F4DD4004BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA6CD55-13B1-40A9-ADDE-A4CE279B69CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Topic Wise" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="151">
   <si>
     <t>Git Commands</t>
   </si>
@@ -223,12 +224,689 @@
 In layman's term:
 git clone is downloading and git pull is refreshing.</t>
   </si>
+  <si>
+    <t>GIT Basics</t>
+  </si>
+  <si>
+    <t>Commands</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
+    <t>git init</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suppose we are in  "C:/Users/user/my_project", This command creates a new subdirectory named .git that contains all of your necessary repository files — a
+Git repository skeleton. At this point, nothing in your project is tracked yet. </t>
+  </si>
+  <si>
+    <t>Initializing a Repository in an Existing Directory</t>
+  </si>
+  <si>
+    <t>git clone &lt;url&gt;</t>
+  </si>
+  <si>
+    <t>Cloning an Existing Repository</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If you’re familiar with other VCSs such as Subversion, you’ll notice that the command is "clone" and not "checkout". This is an important distinction — instead of getting just a working copy, Git receives a full copy of nearly all data that the server has. Every version of every file for the history of the project is pulled down by default when you run git clone. In fact, if your server disk gets corrupted, you can often use nearly any of the clones on any client to set the server back to the state it was in when it was cloned (you may lose some server-side hooks and such, but all the versioned data would be there). That creates a directory named libgit2, initializes a .git directory inside it, pulls down all the data for that repository, and checks out a working copy of the latest version. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remember that each file in your working directory can be in one of two states: tracked or
+untracked. Tracked files are files that were in the last snapshot; they can be unmodified, modified,
+or staged. In short, tracked files are files that Git knows about.Untracked files are everything else — any files in your working directory that were not in your last
+snapshot and are not in your staging area. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git status</t>
+  </si>
+  <si>
+    <t>Checking the Status of Your Files</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The main tool you use to determine which files are in which state is the git status command. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git add &lt;filename&gt;</t>
+  </si>
+  <si>
+    <t>In order to begin tracking a new file, you use the command git add. git add is a multipurpose command — you use it to begin tracking new files, to stage files, and to do other things like marking merge-conflicted files as resolved. It may be helpful to think of it more as “add precisely this content to the next commit” rather than “add this file to the project”.</t>
+  </si>
+  <si>
+    <t>1. Tracking New Files
+2. Staging Modified Files</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Often, you’ll have a class of files that you don’t want Git to automatically add or even show you as
+being untracked. These are generally automatically generated files such as log files or files
+produced by your build system. In such cases, you can create a file listing patterns to match them
+named .gitignore. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">git diff </t>
+  </si>
+  <si>
+    <t>Viewing Your Staged and Unstaged Changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git commit</t>
+  </si>
+  <si>
+    <t>Committing Your Changes</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If the git status command is too vague for you — you want to know exactly what you changed, not just which files were changed — you can use the git diff command. you’ll probably use it most often to answer these two questions: What have you changed but not yet staged? And what have you staged that you are about to commit? That command compares what is in your working directory with what is in your staging area. The result tells you the changes you’ve made that you haven’t yet staged. If you want to see what you’ve staged that will go into your next commit, you can use </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>git diff --staged/ git diff --cached</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>. This command compares your staged changes to your last commit. It’s important to note that git diff by itself doesn’t show all changes made since your last commit — only changes that are still unstaged. If you’ve staged all of your changes, git diff will give you no output.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Remember that anything that is still unstaged — any files you have created or modified that you haven’t run git add on since you edited them — won’t go into this commit. They will stay as modified files on your disk. You can see that the default commit message contains the latest output of the git status command commented out and one empty line on top. You can remove these comments and type your commit message, or you can leave them there to help you remember what you’re committing. For an even more explicit reminder of what you’ve modified, you can pass the</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-v</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> option to git commit. Doing so also puts the diff of your change in the editor so you can see exactly what changes you’re committing. Alternatively, you can type your commit message inline with the commit command by specifying it after a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-m</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> flag. Adding the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-a</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> option to the git commit command makes Git automatically stage every file that is already tracked before doing the commit, letting you skip the git add part</t>
+    </r>
+  </si>
+  <si>
+    <t>Examples</t>
+  </si>
+  <si>
+    <t>git clone https://github.com/libgit2/libgit2</t>
+  </si>
+  <si>
+    <t>git add CONTRIBUTING.md</t>
+  </si>
+  <si>
+    <t>1. git commit -m "Story 182: fix benchmarks for speed"
+2.  git commit -a -m 'Add new benchmarks'</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git rm</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">To remove a file from Git, you have to remove it from your tracked files (more accurately, remove it from your staging area) and then commit. The git rm command does that, and also removes the file from your working directory so you don’t see it as an untracked file the next time around. The next time you commit, the file will be gone and no longer tracked. If you modified the file or had already added it to the staging area, you must force the removal with the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-f</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> option. Another useful thing you may want to do is to keep the file in your working tree but remove it from your staging area. In other words, you may want to keep the file on your hard drive but not have Git track it anymore. This is particularly useful if you forgot to add something to your .gitignore file and accidentally staged it, like a large log file or a bunch of .a compiled files. To do this, use the</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> --cached</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> option</t>
+    </r>
+  </si>
+  <si>
+    <t>1.  git rm PROJECTS.md
+2.  git rm --cached README</t>
+  </si>
+  <si>
+    <t>Removing Files</t>
+  </si>
+  <si>
+    <t>git mv file_from file_to</t>
+  </si>
+  <si>
+    <t>Moving Files</t>
+  </si>
+  <si>
+    <t>Unlike many other VCSs, Git doesn’t explicitly track file movement. If you rename a file in Git, no metadata is stored in Git that tells it you renamed the file. If you want to rename a file in Git, you can run something like "git mv README.md README" and it works fine. In fact, if you run something like this and look at the status, you’ll see that Git considers it a renamed file.</t>
+  </si>
+  <si>
+    <t>git mv README.md README</t>
+  </si>
+  <si>
+    <t xml:space="preserve">git log </t>
+  </si>
+  <si>
+    <t>Viewing the Commit History</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">By default, with no arguments, git log lists the commits made in that repository in reverse chronological order; that is, the most recent commits show up first. As you can see, this command lists each commit with its SHA-1 checksum, the author’s name and email, the date written, and the commit message. One of the more helpful options is </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-p</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> or </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>--patch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, which shows the difference (the patch output)
+introduced in each commit. You can also limit the number of log entries displayed, such as using </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>-2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> to show only the last two entries.  if you want to see some abbreviated stats for each commit, you can use the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>--stat</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> option. Another really useful option is </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>--pretty</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. This option changes the log output to formats other than
+the default. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>oneline</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> value for this option prints each commit on a single line, which is useful if you’re looking at a lot of commits. In addition, the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>short</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>full</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>fuller</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> values show the output in roughly the same format but with less or more information, respectively. The most interesting option value is </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>format</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>, which allows you to specify your own log output format. This is especially useful when you’re generating output for machine parsing — because you specify the format explicitly, you know it won’t change with updates to Git.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. git log
+2.  git log -p -2
+3.  git log --stat
+4. git log --pretty=oneline
+5.  git log --pretty=format:"%h - %an, %ar : %s"</t>
+  </si>
+  <si>
+    <t>Undoing Things</t>
+  </si>
+  <si>
+    <t>git commit --amend</t>
+  </si>
+  <si>
+    <t>1. Add Forgotton Files
+2. Change commit message</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">One of the common undos takes place when you commit too early and possibly forget to add some files, or you mess up your commit message. If you want to redo that commit, make the additional changes you forgot, stage them, and commit again using the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>--amend</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> option. This command takes your staging area and uses it for the commit. If you’ve made no changes since your last commit (for instance, you run this command immediately after your previous commit), then your snapshot will look exactly the same, and all you’ll change is your commit message.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">It’s important to understand that when you’re amending your last commit, you’re
+not so much fixing it as replacing it entirely with a new, improved commit that
+pushes the old commit out of the way and puts the new commit in its place.
+Effectively, it’s as if the previous commit never happened, and it won’t show up in
+your repository history. Only amend commits that are still local and have not been pushed somewhere.
+Amending previously pushed commits and force pushing the branch will cause
+problems for your collaborators. </t>
+  </si>
+  <si>
+    <t>Unstaging a Staged File</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git reset HEAD &lt;file&gt;</t>
+  </si>
+  <si>
+    <t>git reset HEAD CONTRIBUTING.md</t>
+  </si>
+  <si>
+    <t>let’s use that advice to unstage the CONTRIBUTING.md file. The command is a bit strange, but it works. The CONTRIBUTING.md file is modified but once again
+unstaged.</t>
+  </si>
+  <si>
+    <t>git checkout -- &lt;file&gt;</t>
+  </si>
+  <si>
+    <t>Unmodifying a Modified File</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What if you realize that you don’t want to keep your changes to the CONTRIBUTING.md file? How can you easily unmodify it — revert it back to what it looked like when you last committed (or initially cloned, or however you got it into your working directory)? Luckily, git status tells you how to do that, too. </t>
+  </si>
+  <si>
+    <t>git checkout -- CONTRIBUTING.md</t>
+  </si>
+  <si>
+    <t>Remember, anything that is committed in Git can almost always be recovered. Even commits that
+were on branches that were deleted or commits that were overwritten with an --amend commit can
+be recovered (see Data Recovery for data recovery). However, anything you lose that was never
+committed is likely never to be seen again.</t>
+  </si>
+  <si>
+    <t>Unstaging a Staged File with git restore</t>
+  </si>
+  <si>
+    <t>git restore --staged &lt;file&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git restore --staged CONTRIBUTING.md</t>
+  </si>
+  <si>
+    <t>Unmodifying a Modified File with git restore</t>
+  </si>
+  <si>
+    <t>use git restore --staged &lt;file&gt;… to unstage. So, let’s use that advice to unstage the CONTRIBUTING.md fileThe CONTRIBUTING.md file is modified but once again unstaged.</t>
+  </si>
+  <si>
+    <t>git restore &lt;file&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What if you realize that you don’t want to keep your changes to the CONTRIBUTING.md file? How can you easily unmodify it — revert it back to what it looked like when you last committed (or initially cloned, or however you got it into your working directory)? Git just replaced that file with the last staged or committed version. </t>
+  </si>
+  <si>
+    <t>git restore CONTRIBUTING.md</t>
+  </si>
+  <si>
+    <t>Working with Remotes</t>
+  </si>
+  <si>
+    <t>Showing Your Remotes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git remote</t>
+  </si>
+  <si>
+    <r>
+      <t>To see which remote servers you have configured, you can run the git remote command. It lists the shortnames of each remote handle you’ve specified. You can also specify</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> -v</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>, which shows you the URLs that Git has stored for the shortname to be used when reading and writing to that remote.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve"> git remote -v</t>
+  </si>
+  <si>
+    <t>Adding Remote Repositories</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git remote add &lt;shortname&gt; &lt;url&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git remote add pb https://github.com/paulboone/ticgit</t>
+  </si>
+  <si>
+    <t>Now you can use the string pb on the command line in lieu of the whole URL. For example, if you want to fetch all the information that Paul has but that you don’t yet have in your repository, you can run git fetch pb.</t>
+  </si>
+  <si>
+    <t>git fetch &lt;remote&gt;</t>
+  </si>
+  <si>
+    <t>Fetching from Your Remotes</t>
+  </si>
+  <si>
+    <t>The command goes out to that remote project and pulls down all the data from that remote project that you don’t have yet. After you do this, you should have references to all the branches from that remote, which you can merge in or inspect at any time. If you clone a repository, the command automatically adds that remote repository under the name “origin”. So, git fetch origin fetches any new work that has been pushed to that server since you cloned (or last fetched from) it. It’s important to note that the git fetch command only downloads the data to your local repository — it doesn’t automatically merge it with any of your work or modify what you’re currently working on. You have to merge it manually into your work when you’re ready.</t>
+  </si>
+  <si>
+    <t>git pull</t>
+  </si>
+  <si>
+    <t>pulling from Your Remotes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If your current branch is set up to track a remote branch, you can use the git pull command to automatically fetch and then merge that remote branch into your current branch. </t>
+  </si>
+  <si>
+    <t>Pushing to Your Remotes</t>
+  </si>
+  <si>
+    <t>git push &lt;remote&gt; &lt;branch&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If you want to push your master branch to your origin server (again, cloning generally sets up both of those names for you automatically), then you can run this to push any commits you’ve done back up to the server -  git push origin master. If you and someone else clone at the same time and they push upstream and then you push upstream, your push will rightly be rejected. You’ll have to fetch their work first and incorporate it into yours before you’ll be allowed to push. </t>
+  </si>
+  <si>
+    <t>Inspecting a Remote</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git remote show
+&lt;remote&gt;</t>
+  </si>
+  <si>
+    <t>It lists the URL for the remote repository as well as the tracking branch information. The command helpfully tells you that if you’re on the master branch and you run git pull, it will automatically merge the remote’s master branch into the local one after it has been fetched. It also lists all the remote references it has pulled down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git remote rename</t>
+  </si>
+  <si>
+    <t>You can run git remote rename to change a remote’s shortname. It’s worth mentioning that this changes all your remote-tracking branch names, too. What used to be referenced at pb/master is now at paul/master.</t>
+  </si>
+  <si>
+    <t>Renaming Remotes</t>
+  </si>
+  <si>
+    <t>git remote remove</t>
+  </si>
+  <si>
+    <t>Removing Remotes</t>
+  </si>
+  <si>
+    <t>If you want to remove a remote for some reason — you’ve moved the server or are no longer using a particular mirror, or perhaps a contributor isn’t contributing anymore.  Once you delete the reference to a remote this way, all remote-tracking branches and configuration settings associated with that remote are also deleted.</t>
+  </si>
+  <si>
+    <t>Git Aliases</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -243,8 +921,49 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF002060"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -255,6 +974,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8FC6E"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -286,11 +1023,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -311,6 +1045,32 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -387,6 +1147,9 @@
       <rgbColor rgb="00333399"/>
       <rgbColor rgb="00333333"/>
     </indexedColors>
+    <mruColors>
+      <color rgb="FFB8FC6E"/>
+    </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -397,6 +1160,161 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4084320</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90DCA63B-C095-B3D9-CC31-04A2D0E97412}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2293620" y="5615940"/>
+          <a:ext cx="7772400" cy="3352800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>4701540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>3185160</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>256405</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65CF6CC3-08E6-F464-2EE6-2CE6DDC89944}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1394460" y="28704540"/>
+          <a:ext cx="7772400" cy="5422765"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>3154680</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>4351020</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>72801</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43812751-8E9E-4E49-BC14-39242291BC78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9136380" y="28354020"/>
+          <a:ext cx="7772400" cy="4256181"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -699,254 +1617,254 @@
   <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="75.21875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="60.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="163.5546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="75.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="60.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="163.5546875" style="1" customWidth="1"/>
     <col min="4" max="1025" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1"/>
+      <c r="C4" s="9"/>
     </row>
     <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
+    <row r="20" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="B26" s="9" t="s">
+    <row r="26" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="B26" s="8" t="s">
         <v>61</v>
       </c>
     </row>
@@ -957,4 +1875,986 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FAA66C5-738A-4CC1-A5EB-DE4CE7B7410E}">
+  <dimension ref="A1:O93"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="28.44140625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="11"/>
+    <col min="3" max="3" width="24.44140625" style="12" customWidth="1"/>
+    <col min="4" max="4" width="33.6640625" style="12" customWidth="1"/>
+    <col min="5" max="5" width="102.33203125" style="12" customWidth="1"/>
+    <col min="6" max="6" width="17.109375" style="12" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="C1" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2" s="14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="63" x14ac:dyDescent="0.4">
+      <c r="B3" s="11">
+        <v>1</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="210" x14ac:dyDescent="0.4">
+      <c r="B4" s="11">
+        <v>2</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+    </row>
+    <row r="25" spans="2:6" ht="42" x14ac:dyDescent="0.4">
+      <c r="B25" s="11">
+        <v>3</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="105" x14ac:dyDescent="0.4">
+      <c r="B26" s="11">
+        <v>4</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B28" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+    </row>
+    <row r="33" spans="2:15" ht="252" x14ac:dyDescent="0.4">
+      <c r="B33" s="11">
+        <v>5</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="2:15" ht="273" x14ac:dyDescent="0.4">
+      <c r="B34" s="11">
+        <v>6</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="35" spans="2:15" ht="252" x14ac:dyDescent="0.4">
+      <c r="B35" s="11">
+        <v>7</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="2:15" ht="105" x14ac:dyDescent="0.4">
+      <c r="B36" s="11">
+        <v>8</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" spans="2:15" ht="378" x14ac:dyDescent="0.4">
+      <c r="B37" s="11">
+        <v>9</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15"/>
+      <c r="L38" s="15"/>
+      <c r="M38" s="15"/>
+      <c r="N38" s="15"/>
+      <c r="O38" s="15"/>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="15"/>
+      <c r="K39" s="15"/>
+      <c r="L39" s="15"/>
+      <c r="M39" s="15"/>
+      <c r="N39" s="15"/>
+      <c r="O39" s="15"/>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15"/>
+      <c r="L40" s="15"/>
+      <c r="M40" s="15"/>
+      <c r="N40" s="15"/>
+      <c r="O40" s="15"/>
+    </row>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="15"/>
+      <c r="L41" s="15"/>
+      <c r="M41" s="15"/>
+      <c r="N41" s="15"/>
+      <c r="O41" s="15"/>
+    </row>
+    <row r="42" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="15"/>
+      <c r="I42" s="15"/>
+      <c r="J42" s="15"/>
+      <c r="K42" s="15"/>
+      <c r="L42" s="15"/>
+      <c r="M42" s="15"/>
+      <c r="N42" s="15"/>
+      <c r="O42" s="15"/>
+    </row>
+    <row r="43" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
+      <c r="I43" s="15"/>
+      <c r="J43" s="15"/>
+      <c r="K43" s="15"/>
+      <c r="L43" s="15"/>
+      <c r="M43" s="15"/>
+      <c r="N43" s="15"/>
+      <c r="O43" s="15"/>
+    </row>
+    <row r="44" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
+      <c r="I44" s="15"/>
+      <c r="J44" s="15"/>
+      <c r="K44" s="15"/>
+      <c r="L44" s="15"/>
+      <c r="M44" s="15"/>
+      <c r="N44" s="15"/>
+      <c r="O44" s="15"/>
+    </row>
+    <row r="45" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="15"/>
+      <c r="H45" s="15"/>
+      <c r="I45" s="15"/>
+      <c r="J45" s="15"/>
+      <c r="K45" s="15"/>
+      <c r="L45" s="15"/>
+      <c r="M45" s="15"/>
+      <c r="N45" s="15"/>
+      <c r="O45" s="15"/>
+    </row>
+    <row r="46" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
+      <c r="K46" s="15"/>
+      <c r="L46" s="15"/>
+      <c r="M46" s="15"/>
+      <c r="N46" s="15"/>
+      <c r="O46" s="15"/>
+    </row>
+    <row r="47" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15"/>
+      <c r="K47" s="15"/>
+      <c r="L47" s="15"/>
+      <c r="M47" s="15"/>
+      <c r="N47" s="15"/>
+      <c r="O47" s="15"/>
+    </row>
+    <row r="48" spans="2:15" x14ac:dyDescent="0.4">
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
+      <c r="M48" s="15"/>
+      <c r="N48" s="15"/>
+      <c r="O48" s="15"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B49" s="15"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="15"/>
+      <c r="E49" s="15"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="15"/>
+      <c r="H49" s="15"/>
+      <c r="I49" s="15"/>
+      <c r="J49" s="15"/>
+      <c r="K49" s="15"/>
+      <c r="L49" s="15"/>
+      <c r="M49" s="15"/>
+      <c r="N49" s="15"/>
+      <c r="O49" s="15"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
+      <c r="H50" s="15"/>
+      <c r="I50" s="15"/>
+      <c r="J50" s="15"/>
+      <c r="K50" s="15"/>
+      <c r="L50" s="15"/>
+      <c r="M50" s="15"/>
+      <c r="N50" s="15"/>
+      <c r="O50" s="15"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B51" s="15"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+      <c r="H51" s="15"/>
+      <c r="I51" s="15"/>
+      <c r="J51" s="15"/>
+      <c r="K51" s="15"/>
+      <c r="L51" s="15"/>
+      <c r="M51" s="15"/>
+      <c r="N51" s="15"/>
+      <c r="O51" s="15"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="15"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="15"/>
+      <c r="H52" s="15"/>
+      <c r="I52" s="15"/>
+      <c r="J52" s="15"/>
+      <c r="K52" s="15"/>
+      <c r="L52" s="15"/>
+      <c r="M52" s="15"/>
+      <c r="N52" s="15"/>
+      <c r="O52" s="15"/>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="15"/>
+      <c r="I53" s="15"/>
+      <c r="J53" s="15"/>
+      <c r="K53" s="15"/>
+      <c r="L53" s="15"/>
+      <c r="M53" s="15"/>
+      <c r="N53" s="15"/>
+      <c r="O53" s="15"/>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
+      <c r="I54" s="15"/>
+      <c r="J54" s="15"/>
+      <c r="K54" s="15"/>
+      <c r="L54" s="15"/>
+      <c r="M54" s="15"/>
+      <c r="N54" s="15"/>
+      <c r="O54" s="15"/>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
+      <c r="H55" s="15"/>
+      <c r="I55" s="15"/>
+      <c r="J55" s="15"/>
+      <c r="K55" s="15"/>
+      <c r="L55" s="15"/>
+      <c r="M55" s="15"/>
+      <c r="N55" s="15"/>
+      <c r="O55" s="15"/>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
+      <c r="I56" s="15"/>
+      <c r="J56" s="15"/>
+      <c r="K56" s="15"/>
+      <c r="L56" s="15"/>
+      <c r="M56" s="15"/>
+      <c r="N56" s="15"/>
+      <c r="O56" s="15"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B57" s="15"/>
+      <c r="C57" s="15"/>
+      <c r="D57" s="15"/>
+      <c r="E57" s="15"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="15"/>
+      <c r="H57" s="15"/>
+      <c r="I57" s="15"/>
+      <c r="J57" s="15"/>
+      <c r="K57" s="15"/>
+      <c r="L57" s="15"/>
+      <c r="M57" s="15"/>
+      <c r="N57" s="15"/>
+      <c r="O57" s="15"/>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15"/>
+      <c r="F58" s="15"/>
+      <c r="G58" s="15"/>
+      <c r="H58" s="15"/>
+      <c r="I58" s="15"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="15"/>
+      <c r="L58" s="15"/>
+      <c r="M58" s="15"/>
+      <c r="N58" s="15"/>
+      <c r="O58" s="15"/>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A59" s="14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" ht="168" x14ac:dyDescent="0.4">
+      <c r="B60" s="11">
+        <v>1</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="E60" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B62" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C62" s="16"/>
+      <c r="D62" s="16"/>
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B65" s="16"/>
+      <c r="C65" s="16"/>
+      <c r="D65" s="16"/>
+      <c r="E65" s="16"/>
+      <c r="F65" s="16"/>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B66" s="16"/>
+      <c r="C66" s="16"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+    </row>
+    <row r="67" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B67" s="16"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B68" s="16"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+    </row>
+    <row r="69" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B69" s="16"/>
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+    </row>
+    <row r="71" spans="2:6" ht="84" x14ac:dyDescent="0.4">
+      <c r="B71" s="11">
+        <v>2</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="F71" s="12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" ht="84" x14ac:dyDescent="0.4">
+      <c r="B72" s="11">
+        <v>3</v>
+      </c>
+      <c r="C72" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D72" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="E72" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="F72" s="12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B74" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C74" s="16"/>
+      <c r="D74" s="16"/>
+      <c r="E74" s="16"/>
+      <c r="F74" s="16"/>
+    </row>
+    <row r="75" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B75" s="16"/>
+      <c r="C75" s="16"/>
+      <c r="D75" s="16"/>
+      <c r="E75" s="16"/>
+      <c r="F75" s="16"/>
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B76" s="16"/>
+      <c r="C76" s="16"/>
+      <c r="D76" s="16"/>
+      <c r="E76" s="16"/>
+      <c r="F76" s="16"/>
+    </row>
+    <row r="77" spans="2:6" x14ac:dyDescent="0.4">
+      <c r="B77" s="16"/>
+      <c r="C77" s="16"/>
+      <c r="D77" s="16"/>
+      <c r="E77" s="16"/>
+      <c r="F77" s="16"/>
+    </row>
+    <row r="79" spans="2:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B79" s="11">
+        <v>4</v>
+      </c>
+      <c r="C79" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="D79" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="E79" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="F79" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6" ht="105" x14ac:dyDescent="0.4">
+      <c r="B80" s="11">
+        <v>5</v>
+      </c>
+      <c r="C80" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D80" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E80" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="F80" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A82" s="14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="84" x14ac:dyDescent="0.4">
+      <c r="B83" s="11">
+        <v>1</v>
+      </c>
+      <c r="C83" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D83" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="E83" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F83" s="12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" s="17" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A84" s="11"/>
+      <c r="B84" s="11">
+        <v>2</v>
+      </c>
+      <c r="C84" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="D84" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="E84" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="F84" s="12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B85" s="11">
+        <v>3</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="D85" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="E85" s="12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="63" x14ac:dyDescent="0.4">
+      <c r="B86" s="11">
+        <v>4</v>
+      </c>
+      <c r="C86" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D86" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E86" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="147" x14ac:dyDescent="0.4">
+      <c r="B87" s="11">
+        <v>5</v>
+      </c>
+      <c r="C87" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="D87" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="E87" s="12" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="105" x14ac:dyDescent="0.4">
+      <c r="B88" s="11">
+        <v>6</v>
+      </c>
+      <c r="C88" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="D88" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="E88" s="12" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B89" s="11">
+        <v>7</v>
+      </c>
+      <c r="C89" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D89" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="E89" s="12" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="105" x14ac:dyDescent="0.4">
+      <c r="B90" s="11">
+        <v>8</v>
+      </c>
+      <c r="C90" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="D90" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="E90" s="12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A92" s="14" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B93" s="11">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B74:F77"/>
+    <mergeCell ref="B6:F10"/>
+    <mergeCell ref="B28:F31"/>
+    <mergeCell ref="B62:F69"/>
+    <mergeCell ref="B38:O58"/>
+    <mergeCell ref="B11:E23"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>